<commit_message>
cox 결측치 제거 update
</commit_message>
<xml_diff>
--- a/result/FAT1_LUAD_Tables.xlsx
+++ b/result/FAT1_LUAD_Tables.xlsx
@@ -1677,7 +1677,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1714,17 +1714,17 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1.008</v>
+        <v>1.007</v>
       </c>
       <c r="C2" t="n">
-        <v>0.987</v>
+        <v>0.988</v>
       </c>
       <c r="D2" t="n">
-        <v>1.028</v>
+        <v>1.027</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>0.468</t>
+          <t>0.462</t>
         </is>
       </c>
     </row>
@@ -1735,7 +1735,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1</v>
+        <v>1.001</v>
       </c>
       <c r="C3" t="n">
         <v>0.993</v>
@@ -1745,196 +1745,70 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>0.911</t>
+          <t>0.837</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>KrasExpression</t>
+          <t>pathologic_stage</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1</v>
+        <v>1.527</v>
       </c>
       <c r="C4" t="n">
-        <v>1</v>
+        <v>1.28</v>
       </c>
       <c r="D4" t="n">
-        <v>1</v>
+        <v>1.823</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>0.104</t>
+          <t>&lt;0.001</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>TP53Expression</t>
+          <t>FAT1group_Low</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1</v>
+        <v>0.6820000000000001</v>
       </c>
       <c r="C5" t="n">
-        <v>1</v>
+        <v>0.465</v>
       </c>
       <c r="D5" t="n">
         <v>1</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>0.316</t>
+          <t>0.050</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ALKExpression</t>
+          <t>gender_MALE</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.993</v>
+        <v>1.277</v>
       </c>
       <c r="C6" t="n">
-        <v>0.983</v>
+        <v>0.873</v>
       </c>
       <c r="D6" t="n">
-        <v>1.004</v>
+        <v>1.868</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>0.219</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>BRAFExpression</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>0.998</v>
-      </c>
-      <c r="C7" t="n">
-        <v>0.996</v>
-      </c>
-      <c r="D7" t="n">
-        <v>1.001</v>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>0.138</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>FAT1group_Low</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>0.676</v>
-      </c>
-      <c r="C8" t="n">
-        <v>0.452</v>
-      </c>
-      <c r="D8" t="n">
-        <v>1.012</v>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>0.057</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>gender_MALE</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>1.298</v>
-      </c>
-      <c r="C9" t="n">
-        <v>0.873</v>
-      </c>
-      <c r="D9" t="n">
-        <v>1.929</v>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>0.197</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>pathologic_stage_2.0</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>1.991</v>
-      </c>
-      <c r="C10" t="n">
-        <v>1.247</v>
-      </c>
-      <c r="D10" t="n">
-        <v>3.181</v>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>0.004</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>pathologic_stage_3.0</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>2.903</v>
-      </c>
-      <c r="C11" t="n">
-        <v>1.805</v>
-      </c>
-      <c r="D11" t="n">
-        <v>4.67</v>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>&lt;0.001</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>pathologic_stage_4.0</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>2.744</v>
-      </c>
-      <c r="C12" t="n">
-        <v>1.339</v>
-      </c>
-      <c r="D12" t="n">
-        <v>5.624</v>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>0.006</t>
+          <t>0.208</t>
         </is>
       </c>
     </row>

</xml_diff>